<commit_message>
tweak GFCR report shape
</commit_message>
<xml_diff>
--- a/src/api/reports/templates/gfcr.xlsx
+++ b/src/api/reports/templates/gfcr.xlsx
@@ -397,32 +397,32 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Sub-Indicator Name</t>
+          <t>Sub-indicator name</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Area (km2)</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Suggested Citation</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -3443,67 +3443,47 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Facility/solution type</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Business / Finance Solution</t>
+          <t>Facility/solution name</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Sustainable Finance Mechanisms</t>
+          <t>Revenue type</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>Sector</t>
+          <t>Sustainable revenue stream</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>Geographical Coverage</t>
+          <t>Revenue amount</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>Name of TAF (incubator)</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Number of solutions supported by</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Revenue Type</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Sustainable Revenue Source</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Revenue Amount</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -6496,7 +6476,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AA1011"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="28.38" customWidth="1" style="12" min="1" max="1"/>
@@ -6527,579 +6507,579 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customFormat="1" customHeight="1" s="4">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>FinanceColumnName</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Tabs</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Options</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2" ht="25.5" customHeight="1" s="12">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
-          <t>F1-F7, FinanceSolutions, Investments, Revenue</t>
+          <t>F1-F7, FacilitiesSolutions, Investments, Revenues</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Name of the project</t>
         </is>
       </c>
-      <c r="D2" s="13" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
     </row>
     <row r="3" ht="25.5" customHeight="1" s="12">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
-          <t>F1-F7, FinanceSolutions, Investments, Revenue</t>
+          <t>F1-F7, FacilitiesSolutions, Investments, Revenues</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
-          <t>Name of the phase/report</t>
+          <t>Name of the target/report</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Phase 1 target, Mid-term target, Final target, Baseline, Mid-year report, End-year report</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="25.5" customHeight="1" s="12">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Data type</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>F1-F7, FacilitiesSolutions, Investments, Revenues</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Whether it is reported data or target</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Report, Target</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1" s="12">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Reporting date</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>F1-F7, FacilitiesSolutions, Investments, Revenues</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>End date of the reporting period</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>month/day/year</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="12.8" customHeight="1" s="12">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sub-indicator name</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>F1-F7</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Name of the GFCR sub-indicator</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>See GFCR M&amp;E Toolkit for details</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="25.5" customHeight="1" s="12">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Start date</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Date on which to start calculating ecological indicators from MERMAID</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>month/day/year</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="25.5" customHeight="1" s="12">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>End date</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Date on which to end calculating ecological indicators from MERMAID</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>month/day/year</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1" s="12">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Facility/solution type</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FacilitiesSolutions, Investments, Revenues</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Type of facility, reef-positive solution, or programmatic co-financing being reported; a separate entry is required for each</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Technical assistance facility (TAF), Conservation trust fund (CTF), Financial facility, Business solution, Financial mechanism solution, Programmatic co-financing</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="76.5" customHeight="1" s="12">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Facility/solution name</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FacilitiesSolutions, Investments, Revenues</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Name of the facility, reef-positive solution, or programmatic co-financing</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="25.5" customHeight="1" s="12">
-      <c r="A4" s="13" t="inlineStr">
+    <row r="11" ht="25.5" customHeight="1" s="12">
+      <c r="A11" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Sector</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
-          <t>F1-F7, FinanceSolutions, Investments, Revenue</t>
+          <t>FacilitiesSolutions</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
-          <t>Year of the report</t>
+          <t>Sector of the solution in this GFCR Program (see Annex 3 of the GFCR M&amp;E Toolkit)</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Circular Economy and Pollution Management - Pollution Mitigation, Circular Economy and Pollution Management - Sustainable Infrastructure, Circular Economy and Pollution Management - Waste Management, Circular Economy and Pollution Management - Other, Sustainable Coastal Development - Coastal Infrastructure, Sustainable Coastal Development - Coral Restoration Revenue Models, Sustainable Coastal Development - Ecotourism, Sustainable Coastal Development - Other, Sustainable Ocean Production - Aquaculture, Sustainable Ocean Production - Fisheries, Sustainable Ocean Production - Mariculture, Sustainable Ocean Production - Marine Biotechnology Products, Sustainable Ocean Production - Other, Sustainable Ocean Production - Sustainable Small-Scale Fisheries</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="25.5" customHeight="1" s="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Geographical coverage</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>FacilitiesSolutions</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Geographical area covered by the Conservation Trust Fund - regions, countries, or subnational marine/coastal areas (CTF type only)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Regional, National, Subnational</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="25.5" customHeight="1" s="12">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Used a TAF (incubator)?</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FacilitiesSolutions</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Whether the facility/solution used a Technical Assistance Facility (TAF) (e.g., incubator) for early-stage support</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Yes, No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="51" customHeight="1" s="12">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GFCR-funded TAF (incubator)?</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FacilitiesSolutions</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Whether the TAF (e.g., incubator) used was funded by GFCR</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Yes, No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15.75" customHeight="1" s="12">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Name of TAF (incubator)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>FacilitiesSolutions</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Name of the Technical Assistance Facility (TAF) (e.g., incubator) supporting this solution; the TAF must also be added as its own entry</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="25.5" customHeight="1" s="12">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Number of solutions supported by</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FacilitiesSolutions</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Total number of business/financial mechanism solutions supported by this facility, GFCR-supported only (TAF type only)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>Integer</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" s="12">
-      <c r="A5" s="13" t="inlineStr">
+    <row r="17" ht="25.5" customHeight="1" s="12">
+      <c r="A17" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Local enterprise</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>F1-F7</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>Whether it is actual data or target</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>actual, target</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="12.8" customHeight="1" s="12">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Sub-Indicator Name</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>F1-F7</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>Name of the GFCR sub-indicator</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>See monitoring &amp; evaluation toolkit for details</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="25.5" customHeight="1" s="12">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Date Start</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>Date on which to start calculating biological indicators from MERMAID</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>month/day/year</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="25.5" customHeight="1" s="12">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Date End</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>Date on which to end calculating biological indicators from MERMAID</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>month/day/year</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15.75" customHeight="1" s="12">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>Business / Finance Solution</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>FinanceSolutions, Investments, Revenue</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>Name of business / finance solution</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="76.5" customHeight="1" s="12">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>FinanceSolutions, Investments, Revenue</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>Sector (choose most appropriate)</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>marine protected areas, coral ecosystem restoration, invasive species management, sustainable fisheries, sustainable mariculture/aquaculture, ecotourism, plastic waste management, coastal agriculture, sewage and waste-water treatment, other land-based pollutants management, green shipping and cruise ships, clean energy, coastal infrastructure, coastal forestry</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="25.5" customHeight="1" s="12">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>Used a TAF (incubator)?</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>FacilitiesSolutions</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
-          <t>Whether a TAF (incubator) was used for the finance solution</t>
+          <t>Whether the solution is a small-to-medium enterprise operating within the GFCR Program's specific location (applies to F9.3)</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
-          <t>yes, no</t>
+          <t>Yes, No</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="25.5" customHeight="1" s="12">
-      <c r="A12" s="13" t="inlineStr">
+    <row r="18" ht="15.75" customHeight="1" s="12">
+      <c r="A18" t="inlineStr">
         <is>
-          <t>Local Enterprise</t>
+          <t>Gender 2X criteria</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
-          <t>FinanceSolutions</t>
+          <t>FacilitiesSolutions</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
-          <t>Whether or not the finance solution is a local enterprise</t>
+          <t>Whether the solution qualifies under at least one 2X Challenge Criterion (applies to F10)</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
-          <t>yes, no</t>
+          <t>Yes, No</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="25.5" customHeight="1" s="12">
-      <c r="A13" s="13" t="inlineStr">
+    <row r="19" ht="63.75" customHeight="1" s="12">
+      <c r="A19" t="inlineStr">
         <is>
-          <t>Gender Smart Investment</t>
+          <t>Sustainable financial mechanisms</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
-          <t>FinanceSolutions</t>
+          <t>FacilitiesSolutions</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
-          <t>Whether the finance solution represents a gender-smart investment</t>
+          <t>Financial mechanism(s) generating a recurring revenue stream directed toward conservation or sustainable ecosystem management (applies to F8.5); select all that apply</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
-          <t>yes, no</t>
+          <t>Biodiversity credits, Blue bonds, Blue carbon credits, Debt conversion, Economic instruments (fines, penalties, taxes, subsidies, etc.), Financial guarantees, Insurance products, Microfinance/village savings and loans, MPA entry fees, Pay for success, Resilience credits, Sustainable livelihood mechanisms</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="51" customHeight="1" s="12">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="20" ht="25.5" customHeight="1" s="12">
+      <c r="A20" t="inlineStr">
         <is>
-          <t>Sustainable Finance Mechanisms</t>
+          <t>Investment source</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>FinanceSolutions</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>Types of sustainable finance mechanisms used</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>MPA entry fees, debt conversion, blue bonds, insurance products, blue carbon, conservation trust funds, incubator / technical assistance, sustainable livelihood mechanisms, pay for success, biodiversity offsets</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15.75" customHeight="1" s="12">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Investment Source</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
-          <t>Source of investment</t>
+          <t>Source of the investment, entered separately per source (applies to F8)</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
-          <t>public, private, philanthropic, GFCR</t>
+          <t>GFCR, Philanthropy, Private, Public</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="25.5" customHeight="1" s="12">
-      <c r="A16" s="13" t="inlineStr">
+    <row r="21" ht="15.75" customHeight="1" s="12">
+      <c r="A21" t="inlineStr">
         <is>
-          <t>Investment Type</t>
+          <t>Investment type</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
-          <t>Type of investment/ finance mechanism</t>
+          <t>Type of investment for a single source, entered separately per type (applies to F8)</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
-          <t>equity, concessional loan, commercial loan, grant, public budget, financial guarantee, bond, technical assistance</t>
+          <t>Bond, Commercial loan, Concessional loan, Equity, Financial guarantee, Grant, Technical assistance/in-kind</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="25.5" customHeight="1" s="12">
-      <c r="A17" s="13" t="inlineStr">
+    <row r="22" ht="15.75" customHeight="1" s="12">
+      <c r="A22" t="inlineStr">
         <is>
-          <t>GFCR-funded TAF (incubator)?</t>
+          <t>Investment amount</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
-          <t>Whether a GFCR-funded TAF (incubator) was used</t>
+          <t>Cumulative investment amount in US dollars since the start of the GFCR Program (applies to F8)</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>yes, no</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" s="12">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>Investment Amount</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>Investments</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>Dollar amount of investment</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Dollar value</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="63.75" customHeight="1" s="12">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="23" ht="38.25" customHeight="1" s="12">
+      <c r="A23" t="inlineStr">
         <is>
-          <t>Revenue Type</t>
+          <t>Revenue type</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Revenues</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
-          <t>Type of revenue</t>
+          <t>Type of revenue generated by the facility or solution, entered separately per type (applies to F9.1)</t>
         </is>
       </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
-          <t>interest / investment returns, tourism fees, water tariff, green tax, debt conversion, blue bonds, blue carbon, insurance products, conservation trust funds, incubator / technical assistance, sustainable livelihood mechanisms, product sales, user fees</t>
+          <t>Biodiversity credits, Blue bonds, Blue carbon credits/environmental services, Conservation trust funds, Debt conversion, Ecotourism sales, Fees, tariffs, penalties, and other payments, Green tax, Insurance products, Interest/investment returns (e.g., public, private equity), Natural resource sales (e.g., fisheries or aquaculture), Misc. revenue streams, Other sustainable livelihood mechanisms</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="25.5" customHeight="1" s="12">
-      <c r="A20" s="13" t="inlineStr">
+    <row r="24" ht="15.75" customHeight="1" s="12">
+      <c r="A24" t="inlineStr">
         <is>
-          <t>Sustainable Revenue Source</t>
+          <t>Sustainable revenue stream</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Revenues</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
-          <t>Whether this source of revenue is sustainable</t>
+          <t>Whether the revenue is consistently and predictably generated over the long term, supporting the facility or solution's financial stability (applies to F9.2)</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
-          <t>yes, no</t>
+          <t>Yes, No</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" s="12">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="25" ht="15.75" customHeight="1" s="12">
+      <c r="A25" t="inlineStr">
         <is>
-          <t>Revenue Amount</t>
+          <t>Revenue amount</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Revenues</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
-          <t>Dollar amount of annual revenue</t>
+          <t>Cumulative revenue amount in US dollars since the start of the GFCR Program (applies to F9)</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Dollar value</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1" s="12">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Suggested Citation</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Format to use when citing this project</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="38.25" customHeight="1" s="12">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>FacilitiesSolutions, Investments, Revenues</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Type of finance solution</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Technical assistance facility (TAF), Conservation trust fund (CTF), Financial facility, Business solution, Financial mechanism solution, Programmatic co-financing</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="12">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Geographical Coverage</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>FacilitiesSolutions, Investments, Revenues</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Geographical coverage of the finance solution (CTF only)</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Regional, National, Subnational</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="12">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Name of TAF (incubator)</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>FacilitiesSolutions, Investments, Revenues</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Name of the TAF (incubator) used</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-    </row>
     <row r="26" ht="15.75" customHeight="1" s="12">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Number of solutions supported by</t>
+          <t>Suggested citation</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>FacilitiesSolutions, Investments, Revenues</t>
+          <t>F1-F7, FacilitiesSolutions, Investments, Revenues</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Number of solutions supported by this TAF (TAF type only)</t>
+          <t>Format to use when citing this project data</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Text</t>
         </is>
       </c>
     </row>
@@ -7109,14 +7089,14 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
-          <t>F1-F7, FinanceSolutions, Investments, Revenue</t>
+          <t>F1-F7, FacilitiesSolutions, Investments, Revenues</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
-          <t>Notes entered for each indicator, business / finance solution, investment, or revenue source</t>
+          <t>Notes entered for each indicator, facility &amp; solution, investment, or revenue</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -8105,10 +8085,6 @@
     <row r="1005" ht="15.75" customHeight="1" s="12"/>
     <row r="1006" ht="15.75" customHeight="1" s="12"/>
     <row r="1007" ht="15.75" customHeight="1" s="12"/>
-    <row r="1008"/>
-    <row r="1009"/>
-    <row r="1010"/>
-    <row r="1011"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.5118110236220469" footer="0.5118110236220469"/>
@@ -8122,7 +8098,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:H1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -8147,27 +8123,32 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Sub-Indicator Name</t>
+          <t>Sub-indicator name</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Area (km2) </t>
+          <t>Value</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -11069,7 +11050,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:H1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -11094,17 +11075,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Sub-Indicator Name</t>
+          <t>Sub-indicator name</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
@@ -11115,6 +11096,11 @@
       <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -13992,7 +13978,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:J1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -14018,27 +14004,27 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="6" t="inlineStr">
         <is>
-          <t>Date Start</t>
+          <t>Start date</t>
         </is>
       </c>
       <c r="F1" s="6" t="inlineStr">
         <is>
-          <t>Date End</t>
+          <t>End date</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Sub-Indicator Name</t>
+          <t>Sub-indicator name</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
@@ -14049,6 +14035,11 @@
       <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -18955,7 +18946,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G935"/>
+  <dimension ref="A1:H935"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -18980,17 +18971,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Sub-Indicator Name</t>
+          <t>Sub-indicator name</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
@@ -19001,6 +18992,11 @@
       <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -21884,7 +21880,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:H1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -21909,17 +21905,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Sub-Indicator Name</t>
+          <t>Sub-indicator name</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
@@ -21930,6 +21926,11 @@
       <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -24772,7 +24773,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G922"/>
+  <dimension ref="A1:H922"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -24797,17 +24798,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Sub-Indicator Name</t>
+          <t>Sub-indicator name</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
@@ -24818,6 +24819,11 @@
       <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -27675,7 +27681,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P1000"/>
+  <dimension ref="A1:Q1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -27704,72 +27710,77 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Facility/solution type</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Business / Finance Solution</t>
+          <t>Facility/solution name</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Sustainable Finance Mechanisms</t>
+          <t>Sector</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>Sector</t>
+          <t>Geographical coverage</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>Geographical Coverage</t>
+          <t>Used a TAF (incubator)?</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>Name of TAF (incubator)</t>
+          <t>GFCR-funded TAF (incubator)?</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>Number of solutions supported by</t>
+          <t>Name of TAF (incubator)</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
         <is>
-          <t>Used a TAF (incubator)?</t>
+          <t>Number of solutions supported by</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>GFCR-funded TAF (incubator)?</t>
+          <t>Local enterprise</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Local Enterprise</t>
+          <t>Gender 2X criteria</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Gender Smart Investment</t>
+          <t>Sustainable financial mechanisms</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>
@@ -30791,67 +30802,47 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Reporting Date</t>
+          <t>Data type</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Data Type</t>
+          <t>Reporting date</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Facility/solution type</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Business / Finance Solution</t>
+          <t>Facility/solution name</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Sustainable Finance Mechanisms</t>
+          <t>Investment source</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>Sector</t>
+          <t>Investment type</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>Geographical Coverage</t>
+          <t>Investment amount</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>Name of TAF (incubator)</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>Number of solutions supported by</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Investment Source</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Investment Type</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Investment Amount</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+          <t>Suggested citation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
make gfcr xlsx headers bold
header row on all sheets set to bold Arial 11; no other changes
</commit_message>
<xml_diff>
--- a/src/api/reports/templates/gfcr.xlsx
+++ b/src/api/reports/templates/gfcr.xlsx
@@ -385,12 +385,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
@@ -420,7 +420,7 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -3415,7 +3415,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1000"/>
+  <dimension ref="A1:K1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -3431,7 +3431,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
@@ -3481,7 +3481,7 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -6507,27 +6507,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customFormat="1" customHeight="1" s="4">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>FinanceColumnName</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Tabs</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Options</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -8111,12 +8111,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
@@ -8141,12 +8141,12 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -11063,12 +11063,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
@@ -11093,12 +11093,12 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -13992,12 +13992,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
@@ -14032,12 +14032,12 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -18959,12 +18959,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
@@ -18989,12 +18989,12 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -21893,12 +21893,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
@@ -21923,12 +21923,12 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -24786,12 +24786,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
@@ -24816,12 +24816,12 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -27698,7 +27698,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
@@ -27728,7 +27728,7 @@
           <t>Facility/solution name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
@@ -27753,32 +27753,32 @@
           <t>Name of TAF (incubator)</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Number of solutions supported by</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Local enterprise</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Gender 2X criteria</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Sustainable financial mechanisms</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>
@@ -30774,7 +30774,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1001"/>
+  <dimension ref="A1:K1001"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.7421875" defaultRowHeight="12.75"/>
   <cols>
     <col width="10.38" customWidth="1" style="12" min="1" max="1"/>
@@ -30790,7 +30790,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="12">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
@@ -30840,7 +30840,7 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Suggested citation</t>
         </is>

</xml_diff>